<commit_message>
report has been "implemented" and BW to BSM
</commit_message>
<xml_diff>
--- a/Legacy data vessels.xlsx
+++ b/Legacy data vessels.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AndersEmilBusk\Desktop\New register page test\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AndersEmilBusk\Desktop\MFT_data_handler\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABADF4E1-AA06-44AB-94BC-FC12C4822812}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3BB31A6-7FBB-438A-A087-F38EBD194410}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25510" yWindow="0" windowWidth="25780" windowHeight="13770" xr2:uid="{9994A8F6-3190-471E-B791-9B9DB550B49C}"/>
+    <workbookView xWindow="3040" yWindow="630" windowWidth="25780" windowHeight="13770" xr2:uid="{9994A8F6-3190-471E-B791-9B9DB550B49C}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="614" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="614" uniqueCount="207">
   <si>
     <t>Adriatic Gas</t>
   </si>
@@ -654,6 +654,9 @@
   </si>
   <si>
     <t>WBE + SBO + ABU</t>
+  </si>
+  <si>
+    <t>BSM</t>
   </si>
 </sst>
 </file>
@@ -1819,7 +1822,7 @@
         <v>9674842</v>
       </c>
       <c r="B29" t="s">
-        <v>146</v>
+        <v>206</v>
       </c>
       <c r="C29" t="s">
         <v>27</v>
@@ -1848,7 +1851,7 @@
         <v>9674854</v>
       </c>
       <c r="B30" t="s">
-        <v>146</v>
+        <v>206</v>
       </c>
       <c r="C30" t="s">
         <v>28</v>
@@ -4564,27 +4567,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="e92f16c9-db69-4522-84e2-bf933696a321" xsi:nil="true"/>
-    <_x0031_0 xmlns="6e040d9b-4d00-4c60-b912-ca778ccae294" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="6e040d9b-4d00-4c60-b912-ca778ccae294">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x0101000B73ECAA2334A14EB365ED6608A878E1" ma:contentTypeVersion="20" ma:contentTypeDescription="Opret et nyt dokument." ma:contentTypeScope="" ma:versionID="aa261c57a18327ad4c092a13a9f1b96d">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6e040d9b-4d00-4c60-b912-ca778ccae294" xmlns:ns3="e92f16c9-db69-4522-84e2-bf933696a321" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ada142b233870dd5f0255efd6e0c4bae" ns2:_="" ns3:_="">
     <xsd:import namespace="6e040d9b-4d00-4c60-b912-ca778ccae294"/>
@@ -4851,10 +4833,42 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="e92f16c9-db69-4522-84e2-bf933696a321" xsi:nil="true"/>
+    <_x0031_0 xmlns="6e040d9b-4d00-4c60-b912-ca778ccae294" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="6e040d9b-4d00-4c60-b912-ca778ccae294">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{855F6443-400B-4276-AA3F-D8A900D50BF5}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0E3BECD9-BD61-4DD0-AD49-ADAA4A55C970}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="6e040d9b-4d00-4c60-b912-ca778ccae294"/>
+    <ds:schemaRef ds:uri="e92f16c9-db69-4522-84e2-bf933696a321"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -4871,20 +4885,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0E3BECD9-BD61-4DD0-AD49-ADAA4A55C970}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{855F6443-400B-4276-AA3F-D8A900D50BF5}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="6e040d9b-4d00-4c60-b912-ca778ccae294"/>
-    <ds:schemaRef ds:uri="e92f16c9-db69-4522-84e2-bf933696a321"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>